<commit_message>
fix jhockey image extension
</commit_message>
<xml_diff>
--- a/data/projects.xlsx
+++ b/data/projects.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anwaypimpalkar/everything/anwaypimpalkar-new/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anwaypimpalkar/everything/anwaypimpalkar.github.io/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34CAF33-7171-394E-AADB-BD85C152020D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF8C4C2C-A28D-8540-8107-CB61386FF855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" xr2:uid="{46DB94BC-6658-C940-A428-5CA04B255DCE}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17820" xr2:uid="{46DB94BC-6658-C940-A428-5CA04B255DCE}"/>
   </bookViews>
   <sheets>
     <sheet name="projects" sheetId="1" r:id="rId1"/>
@@ -282,9 +282,6 @@
     <t>robotics;ai</t>
   </si>
   <si>
-    <t>assets/images/publications/JHockey.jpg</t>
-  </si>
-  <si>
     <t>Two mechatronic robots fighting for a hockey puck in an arena.</t>
   </si>
   <si>
@@ -298,6 +295,9 @@
   </si>
   <si>
     <t>Pneumatactors: Soft interface for co-located multimodal tactile stimuli.</t>
+  </si>
+  <si>
+    <t>assets/images/publications/JHockey.jpeg</t>
   </si>
 </sst>
 </file>
@@ -1422,7 +1422,7 @@
         <v>67</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>57</v>
@@ -1473,13 +1473,13 @@
     </row>
     <row r="7" spans="1:12" ht="38" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B7" s="8" t="s">
         <v>29</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>43</v>
@@ -1503,7 +1503,7 @@
       </c>
       <c r="L7" s="9"/>
     </row>
-    <row r="8" spans="1:12" ht="95" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="76" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>46</v>
       </c>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="L9" s="9"/>
     </row>
-    <row r="10" spans="1:12" ht="171" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="152" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>61</v>
       </c>
@@ -1595,7 +1595,7 @@
         <v>65</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H10" s="8"/>
       <c r="I10" s="8" t="s">
@@ -1628,10 +1628,10 @@
         <v>2024</v>
       </c>
       <c r="F11" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="8" t="s">
         <v>81</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>82</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>70</v>

</xml_diff>